<commit_message>
more references added for future expansions
</commit_message>
<xml_diff>
--- a/Lewitus_etal_2014/pbio.1002000.s014.xlsx
+++ b/Lewitus_etal_2014/pbio.1002000.s014.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10211"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10311"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alleninstitute.sharepoint.com/sites/MammalianM1/Shared Documents/General/Species/Evo-M1-Trait-Data/Lewitus_etal_2014/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_20944A8CF0AFB844FF536A1D6C59DA568678326C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_20944A8CF0AFB844FF536A1D6C59DA568678326C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73A69E50-4384-F44A-BFAB-D2DA5EE543C7}"/>
   <bookViews>
-    <workbookView xWindow="42100" yWindow="-7080" windowWidth="15600" windowHeight="21100" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="42100" yWindow="-5960" windowWidth="25700" windowHeight="26800" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1556,24 +1556,45 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="4"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="4"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="4"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="4"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1581,27 +1602,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="4"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="4"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="4"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="4"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1981,21 +1981,21 @@
       <c r="A4" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="32"/>
+      <c r="B4" s="39"/>
       <c r="C4" s="8" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="26" x14ac:dyDescent="0.2">
-      <c r="A5" s="31"/>
-      <c r="B5" s="33"/>
+      <c r="A5" s="26"/>
+      <c r="B5" s="40"/>
       <c r="C5" s="8" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="26"/>
-      <c r="B6" s="34"/>
+      <c r="A6" s="27"/>
+      <c r="B6" s="41"/>
       <c r="C6" s="9" t="s">
         <v>10</v>
       </c>
@@ -2004,33 +2004,33 @@
       <c r="A7" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="35" t="s">
+      <c r="B7" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="37" t="s">
+      <c r="C7" s="33" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="26"/>
-      <c r="B8" s="36"/>
-      <c r="C8" s="38"/>
+      <c r="A8" s="27"/>
+      <c r="B8" s="32"/>
+      <c r="C8" s="34"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="27" t="s">
+      <c r="B9" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="39" t="s">
+      <c r="C9" s="35" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="26"/>
-      <c r="B10" s="28"/>
-      <c r="C10" s="40"/>
+      <c r="A10" s="27"/>
+      <c r="B10" s="30"/>
+      <c r="C10" s="36"/>
     </row>
     <row r="11" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
@@ -2047,30 +2047,30 @@
       <c r="A12" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="27" t="s">
+      <c r="B12" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="39" t="s">
+      <c r="C12" s="35" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="26"/>
-      <c r="B13" s="28"/>
-      <c r="C13" s="40"/>
+      <c r="A13" s="27"/>
+      <c r="B13" s="30"/>
+      <c r="C13" s="36"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="B14" s="35"/>
+      <c r="B14" s="31"/>
       <c r="C14" s="12" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="26"/>
-      <c r="B15" s="36"/>
+      <c r="A15" s="27"/>
+      <c r="B15" s="32"/>
       <c r="C15" s="13" t="s">
         <v>20</v>
       </c>
@@ -2079,55 +2079,55 @@
       <c r="A16" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="B16" s="27" t="s">
+      <c r="B16" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="C16" s="29" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="26"/>
-      <c r="B17" s="28"/>
-      <c r="C17" s="30"/>
+      <c r="C16" s="37" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="81" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="27"/>
+      <c r="B17" s="30"/>
+      <c r="C17" s="38"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="B18" s="35" t="s">
+      <c r="B18" s="31" t="s">
         <v>24</v>
       </c>
-      <c r="C18" s="37" t="s">
+      <c r="C18" s="33" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="26"/>
-      <c r="B19" s="36"/>
-      <c r="C19" s="38"/>
+      <c r="A19" s="27"/>
+      <c r="B19" s="32"/>
+      <c r="C19" s="34"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="B20" s="27" t="s">
+      <c r="B20" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="39" t="s">
+      <c r="C20" s="35" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="26"/>
-      <c r="B21" s="28"/>
-      <c r="C21" s="40"/>
+      <c r="A21" s="27"/>
+      <c r="B21" s="30"/>
+      <c r="C21" s="36"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="B22" s="27" t="s">
+      <c r="B22" s="28" t="s">
         <v>27</v>
       </c>
       <c r="C22" s="14" t="s">
@@ -2135,50 +2135,50 @@
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A23" s="31"/>
-      <c r="B23" s="41"/>
+      <c r="A23" s="26"/>
+      <c r="B23" s="29"/>
       <c r="C23" s="14" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A24" s="31"/>
-      <c r="B24" s="41"/>
+      <c r="A24" s="26"/>
+      <c r="B24" s="29"/>
       <c r="C24" s="14" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A25" s="31"/>
-      <c r="B25" s="41"/>
+      <c r="A25" s="26"/>
+      <c r="B25" s="29"/>
       <c r="C25" s="14" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A26" s="31"/>
-      <c r="B26" s="41"/>
+      <c r="A26" s="26"/>
+      <c r="B26" s="29"/>
       <c r="C26" s="14" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A27" s="31"/>
-      <c r="B27" s="41"/>
+      <c r="A27" s="26"/>
+      <c r="B27" s="29"/>
       <c r="C27" s="14" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A28" s="31"/>
-      <c r="B28" s="41"/>
+      <c r="A28" s="26"/>
+      <c r="B28" s="29"/>
       <c r="C28" s="14" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="26"/>
-      <c r="B29" s="28"/>
+      <c r="A29" s="27"/>
+      <c r="B29" s="30"/>
       <c r="C29" s="15" t="s">
         <v>35</v>
       </c>
@@ -2249,7 +2249,7 @@
       <c r="A36" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="B36" s="27" t="s">
+      <c r="B36" s="28" t="s">
         <v>44</v>
       </c>
       <c r="C36" s="17" t="s">
@@ -2257,22 +2257,22 @@
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A37" s="31"/>
-      <c r="B37" s="41"/>
+      <c r="A37" s="26"/>
+      <c r="B37" s="29"/>
       <c r="C37" s="17" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A38" s="31"/>
-      <c r="B38" s="41"/>
+      <c r="A38" s="26"/>
+      <c r="B38" s="29"/>
       <c r="C38" s="17" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="26"/>
-      <c r="B39" s="28"/>
+      <c r="A39" s="27"/>
+      <c r="B39" s="30"/>
       <c r="C39" s="18" t="s">
         <v>48</v>
       </c>
@@ -2435,28 +2435,28 @@
       <c r="A54" s="25" t="s">
         <v>69</v>
       </c>
-      <c r="B54" s="27"/>
+      <c r="B54" s="28"/>
       <c r="C54" s="14" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A55" s="31"/>
-      <c r="B55" s="41"/>
+      <c r="A55" s="26"/>
+      <c r="B55" s="29"/>
       <c r="C55" s="14" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A56" s="31"/>
-      <c r="B56" s="41"/>
+      <c r="A56" s="26"/>
+      <c r="B56" s="29"/>
       <c r="C56" s="14" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="57" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="26"/>
-      <c r="B57" s="28"/>
+      <c r="A57" s="27"/>
+      <c r="B57" s="30"/>
       <c r="C57" s="15" t="s">
         <v>73</v>
       </c>
@@ -2465,21 +2465,21 @@
       <c r="A58" s="25" t="s">
         <v>74</v>
       </c>
-      <c r="B58" s="27"/>
+      <c r="B58" s="28"/>
       <c r="C58" s="19" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A59" s="31"/>
-      <c r="B59" s="41"/>
+      <c r="A59" s="26"/>
+      <c r="B59" s="29"/>
       <c r="C59" s="20" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="60" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="26"/>
-      <c r="B60" s="28"/>
+      <c r="A60" s="27"/>
+      <c r="B60" s="30"/>
       <c r="C60" s="21" t="s">
         <v>77</v>
       </c>
@@ -2519,20 +2519,6 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="A58:A60"/>
-    <mergeCell ref="B58:B60"/>
-    <mergeCell ref="A22:A29"/>
-    <mergeCell ref="B22:B29"/>
-    <mergeCell ref="A36:A39"/>
-    <mergeCell ref="B36:B39"/>
-    <mergeCell ref="A54:A57"/>
-    <mergeCell ref="B54:B57"/>
-    <mergeCell ref="A18:A19"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:C21"/>
     <mergeCell ref="A16:A17"/>
     <mergeCell ref="B16:B17"/>
     <mergeCell ref="C16:C17"/>
@@ -2549,6 +2535,20 @@
     <mergeCell ref="C12:C13"/>
     <mergeCell ref="A14:A15"/>
     <mergeCell ref="B14:B15"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="A58:A60"/>
+    <mergeCell ref="B58:B60"/>
+    <mergeCell ref="A22:A29"/>
+    <mergeCell ref="B22:B29"/>
+    <mergeCell ref="A36:A39"/>
+    <mergeCell ref="B36:B39"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="B54:B57"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <extLst>
@@ -2560,6 +2560,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009B0162F312A93D41AE706303C1572F17" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="66af2654134d243f62aac8e2b322f1d6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8e1efd23-f4ba-42d2-85fd-6a510437bae6" xmlns:ns3="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2bc3adf68671d86faa9c37249f400344" ns2:_="" ns3:_="">
     <xsd:import namespace="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
@@ -2802,16 +2811,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1C573D47-6997-49C7-90CC-73CF66448ABB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{73CD1619-5447-4119-9ECF-711B762BD938}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2828,12 +2836,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1C573D47-6997-49C7-90CC-73CF66448ABB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>